<commit_message>
Fix H→G refs: TEMPLATE FONDO LIQUIDEZ ACTIVA.xlsx
</commit_message>
<xml_diff>
--- a/inputs/templates/TEMPLATE FONDO LIQUIDEZ ACTIVA.xlsx
+++ b/inputs/templates/TEMPLATE FONDO LIQUIDEZ ACTIVA.xlsx
@@ -2087,7 +2087,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CL"/>
           </a:p>
@@ -2139,7 +2139,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CL"/>
           </a:p>
@@ -2224,7 +2224,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="es-CL"/>
         </a:p>
@@ -2628,7 +2628,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t/>
+                <a:t>None</a:t>
               </a:r>
               <a:endParaRPr lang="es-CL"/>
             </a:p>
@@ -2660,7 +2660,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CL"/>
           </a:p>
@@ -2697,7 +2697,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="es-CL"/>
         </a:p>
@@ -6167,15 +6167,15 @@
         <v/>
       </c>
       <c r="Y31" s="118">
-        <f>+H183</f>
+        <f>+G183</f>
         <v/>
       </c>
       <c r="Z31" s="118">
-        <f>+H184</f>
+        <f>+G184</f>
         <v/>
       </c>
       <c r="AA31" s="118">
-        <f>+H185</f>
+        <f>+G185</f>
         <v/>
       </c>
       <c r="AD31" s="32" t="n">
@@ -6448,7 +6448,7 @@
         <v>2025</v>
       </c>
       <c r="P36" s="116">
-        <f>+H236</f>
+        <f>+G236</f>
         <v/>
       </c>
       <c r="Q36" s="116">
@@ -6456,43 +6456,43 @@
         <v/>
       </c>
       <c r="R36" s="116">
-        <f>+H236</f>
+        <f>+G236</f>
         <v/>
       </c>
       <c r="S36" s="116">
-        <f>+H237</f>
+        <f>+G237</f>
         <v/>
       </c>
       <c r="T36" s="116">
-        <f>+H238</f>
+        <f>+G238</f>
         <v/>
       </c>
       <c r="U36" s="116">
-        <f>+H239</f>
+        <f>+G239</f>
         <v/>
       </c>
       <c r="V36" s="116">
-        <f>+H240</f>
+        <f>+G240</f>
         <v/>
       </c>
       <c r="W36" s="116">
-        <f>+H241</f>
+        <f>+G241</f>
         <v/>
       </c>
       <c r="X36" s="116">
-        <f>+H242</f>
+        <f>+G242</f>
         <v/>
       </c>
       <c r="Y36" s="116">
-        <f>+H243</f>
+        <f>+G243</f>
         <v/>
       </c>
       <c r="Z36" s="116">
-        <f>+H244</f>
+        <f>+G244</f>
         <v/>
       </c>
       <c r="AA36" s="116">
-        <f>+H245</f>
+        <f>+G245</f>
         <v/>
       </c>
       <c r="AD36" s="32" t="n">
@@ -6525,23 +6525,23 @@
         <v>2026</v>
       </c>
       <c r="P37" s="116">
-        <f>+H246</f>
+        <f>+G246</f>
         <v/>
       </c>
       <c r="Q37" s="116">
-        <f>+H247</f>
+        <f>+G247</f>
         <v/>
       </c>
       <c r="R37" s="116">
-        <f>+H248</f>
+        <f>+G248</f>
         <v/>
       </c>
       <c r="S37" s="116">
-        <f>+H249</f>
+        <f>+G249</f>
         <v/>
       </c>
       <c r="T37" s="116">
-        <f>+H250</f>
+        <f>+G250</f>
         <v/>
       </c>
       <c r="U37" s="116" t="n"/>

</xml_diff>

<commit_message>
Junio 2026 generado con la planilla (sin ODS)
- Todos los templates avanzados a jun-2026 con VC de planilla_vc.xlsx.
- Fix DIVIDENDOS Recurrente (0.0; 177.5114 era erroneo por RUT heredado).
- Guard en snapshot_usd_frozen: no pisar historico USD bueno con uno vacio/parcial
  (permite historico USD correcto aunque el template quede no-pristino).
- hist_usd_frozen.json regenerado desde templates pristinos.
- inputs planilla_vc.xlsx y cartera.xlsx de junio; folletos/2026-06 (HTML preview).
- 24 folletos OK; RUTs corregidos; retornos validados (Recurrente 0.575%/5.14%).
</commit_message>
<xml_diff>
--- a/inputs/templates/TEMPLATE FONDO LIQUIDEZ ACTIVA.xlsx
+++ b/inputs/templates/TEMPLATE FONDO LIQUIDEZ ACTIVA.xlsx
@@ -3980,7 +3980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK250"/>
+  <dimension ref="A1:BK251"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.28515625" defaultRowHeight="15"/>
   <cols>
     <col width="18.28515625" customWidth="1" style="14" min="1" max="2"/>
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="AW19" s="84" t="n">
-        <v>46173</v>
+        <v>46203</v>
       </c>
       <c r="AX19" s="42">
         <f>EOMONTH($AW19,AX18)+6+1</f>
@@ -5342,7 +5342,10 @@
         <f>+T23/S23-1</f>
         <v/>
       </c>
-      <c r="AJ22" s="20" t="n"/>
+      <c r="AJ22" s="20">
+        <f>+U23/T23-1</f>
+        <v/>
+      </c>
       <c r="AK22" s="20" t="n"/>
       <c r="AL22" s="20" t="n"/>
       <c r="AM22" s="20" t="n"/>
@@ -5350,7 +5353,7 @@
       <c r="AO22" s="20" t="n"/>
       <c r="AP22" s="20" t="n"/>
       <c r="AQ22" s="34">
-        <f>+(T23/P23-1)/COUNTA(AE22:AI22)*12</f>
+        <f>+(U23/P23-1)/COUNTA(AE22:AJ22)*12</f>
         <v/>
       </c>
       <c r="AV22" s="39" t="inlineStr">
@@ -5413,7 +5416,10 @@
         <f>+B250</f>
         <v/>
       </c>
-      <c r="U23" s="30" t="n"/>
+      <c r="U23" s="30">
+        <f>+B251</f>
+        <v/>
+      </c>
       <c r="Y23" s="30" t="n"/>
       <c r="AD23" s="37" t="inlineStr">
         <is>
@@ -6544,7 +6550,10 @@
         <f>+G250</f>
         <v/>
       </c>
-      <c r="U37" s="116" t="n"/>
+      <c r="U37" s="116">
+        <f>+G251</f>
+        <v/>
+      </c>
       <c r="V37" s="116" t="n"/>
       <c r="W37" s="116" t="n"/>
       <c r="X37" s="116" t="n"/>
@@ -6681,8 +6690,12 @@
         <f>+T37/S37-1</f>
         <v/>
       </c>
+      <c r="AJ38">
+        <f>+U37/T37-1</f>
+        <v/>
+      </c>
       <c r="AQ38" s="34">
-        <f>+(T37/P37-1)/COUNTA(AE38:AI38)*12</f>
+        <f>+(U37/P37-1)/COUNTA(AE38:AJ38)*12</f>
         <v/>
       </c>
       <c r="AR38" s="37" t="inlineStr">
@@ -7526,6 +7539,10 @@
         <f>+K250</f>
         <v/>
       </c>
+      <c r="U51">
+        <f>+K251</f>
+        <v/>
+      </c>
       <c r="AD51" s="32" t="n">
         <v>2026</v>
       </c>
@@ -7549,7 +7566,10 @@
         <f>+T51/S51-1</f>
         <v/>
       </c>
-      <c r="AJ51" s="20" t="n"/>
+      <c r="AJ51" s="20">
+        <f>+U51/T51-1</f>
+        <v/>
+      </c>
       <c r="AK51" s="20" t="n"/>
       <c r="AL51" s="20" t="n"/>
       <c r="AM51" s="20" t="n"/>
@@ -7557,7 +7577,7 @@
       <c r="AO51" s="20" t="n"/>
       <c r="AP51" s="20" t="n"/>
       <c r="AQ51" s="34">
-        <f>+(T51/P51-1)/COUNTA(AE51:AI51)*12</f>
+        <f>+(U51/P51-1)/COUNTA(AE51:AJ51)*12</f>
         <v/>
       </c>
       <c r="AR51" s="20" t="n"/>
@@ -14812,6 +14832,51 @@
       </c>
       <c r="M250">
         <f>+M249*(1+L250)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="127" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B251" t="n">
+        <v>26634.69</v>
+      </c>
+      <c r="C251">
+        <f>(B251/B250-1)/(A251-A250)*30</f>
+        <v/>
+      </c>
+      <c r="D251">
+        <f>+D250*(1+C251)</f>
+        <v/>
+      </c>
+      <c r="F251" s="127" t="n">
+        <v>46203</v>
+      </c>
+      <c r="G251" t="n">
+        <v>1082.6699</v>
+      </c>
+      <c r="H251">
+        <f>+G251+$S$148+$S$150+$S$152+$S$154+$S$156+$S$158</f>
+        <v/>
+      </c>
+      <c r="I251">
+        <f>+(H251/H250-1)/(F251-F250)*30</f>
+        <v/>
+      </c>
+      <c r="J251">
+        <f>+J250*(1+I251)</f>
+        <v/>
+      </c>
+      <c r="K251" t="n">
+        <v>6385.6713</v>
+      </c>
+      <c r="L251">
+        <f>+(K251/K250-1)/(F251-F250)*30</f>
+        <v/>
+      </c>
+      <c r="M251">
+        <f>+M250*(1+L251)</f>
         <v/>
       </c>
     </row>

</xml_diff>